<commit_message>
Filtro de solicitante adicionado e correção de formato de valor para BRL R$
</commit_message>
<xml_diff>
--- a/custo_dsv.xlsx
+++ b/custo_dsv.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\custo_dsv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2B459176-93C7-4FE9-A6E9-0676CE4BD188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B02411C2-4660-4A83-8599-7FEECA351B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3690" yWindow="-12510" windowWidth="21600" windowHeight="11175" xr2:uid="{1EAB647C-9F39-455D-AECE-6F7B651A9B58}"/>
+    <workbookView xWindow="0" yWindow="240" windowWidth="19360" windowHeight="10480" xr2:uid="{1EAB647C-9F39-455D-AECE-6F7B651A9B58}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>